<commit_message>
Strip all non-ASCII characters and AI markers for production readiness
- Replaced all em dashes (U+2014) with standard hyphens throughout
  lookup values, comments, dashboard labels, and HOME descriptions
- Replaced all arrow characters (U+2192) with ASCII > equivalents
- Replaced box-drawing section dividers (U+2550) with plain = lines
- Removed AI-sounding docstring language (Purpose-Driven Redesign,
  Built from research, etc.) and replaced with clean institutional text
- Updated version references to v2.1
- Verified zero non-ASCII characters remain in the entire script
- Regenerated workbook from cleaned source

https://claude.ai/code/session_01PQmx3HYDSPG2GvHuVy9J6w
</commit_message>
<xml_diff>
--- a/FNID_Area3_Operational_Workbook.xlsx
+++ b/FNID_Area3_Operational_Workbook.xlsx
@@ -1168,14 +1168,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>JAMAICA CONSTABULARY FORCE — FIREARM AND NARCOTICS INVESTIGATION DIVISION</t>
+          <t>JAMAICA CONSTABULARY FORCE - FIREARM AND NARCOTICS INVESTIGATION DIVISION</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AREA 3 (Manchester | St. Elizabeth | Clarendon) — OPERATIONAL WORKBOOK v2.0</t>
+          <t>AREA 3 (Manchester | St. Elizabeth | Clarendon) - OPERATIONAL WORKBOOK v2.1</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>INTELLIGENCE → OPERATION → SEIZURE → ARREST → FORENSICS → DPP → COURT → CONVICTION</t>
+          <t>INTELLIGENCE &gt; OPERATION &gt; SEIZURE &gt; ARREST &gt; FORENSICS &gt; DPP &gt; COURT &gt; CONVICTION</t>
         </is>
       </c>
     </row>
@@ -1203,12 +1203,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; DASH_Command</t>
+          <t xml:space="preserve">  &gt; DASH_Command</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Daily Command Dashboard — all key metrics at a glance</t>
+          <t>Daily Command Dashboard - all key metrics at a glance</t>
         </is>
       </c>
     </row>
@@ -1222,24 +1222,24 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_IntelLog</t>
+          <t xml:space="preserve">  &gt; tbl_IntelLog</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Intelligence Log — Crime Stop, NIB, DEA, JCA, informant tips</t>
+          <t>Intelligence Log - Crime Stop, NIB, DEA, JCA, informant tips</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_Informants</t>
+          <t xml:space="preserve">  &gt; tbl_Informants</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Informant Register — RESTRICTED ACCESS (code names only)</t>
+          <t>Informant Register - RESTRICTED ACCESS (code names only)</t>
         </is>
       </c>
     </row>
@@ -1253,12 +1253,12 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_Operations</t>
+          <t xml:space="preserve">  &gt; tbl_Operations</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Operation Register — warrants, teams, execution, outcomes</t>
+          <t>Operation Register - warrants, teams, execution, outcomes</t>
         </is>
       </c>
     </row>
@@ -1272,36 +1272,36 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_FirearmSeizures</t>
+          <t xml:space="preserve">  &gt; tbl_FirearmSeizures</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Firearm Seizure Log — IBIS, eTrace, ballistic cert tracking</t>
+          <t>Firearm Seizure Log - IBIS, eTrace, ballistic cert tracking</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_NarcoticSeizures</t>
+          <t xml:space="preserve">  &gt; tbl_NarcoticSeizures</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Narcotics Seizure Log — field test, IFSLM, forensic cert, disposal</t>
+          <t>Narcotics Seizure Log - field test, IFSLM, forensic cert, disposal</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_OtherSeizures</t>
+          <t xml:space="preserve">  &gt; tbl_OtherSeizures</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Ammunition, Cash, Electronics, Vehicles — other exhibits</t>
+          <t>Ammunition, Cash, Electronics, Vehicles - other exhibits</t>
         </is>
       </c>
     </row>
@@ -1315,12 +1315,12 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_Arrests</t>
+          <t xml:space="preserve">  &gt; tbl_Arrests</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Arrest Register — 48hr rule, charge, caution, bail, court routing</t>
+          <t>Arrest Register - 48hr rule, charge, caution, bail, court routing</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_CaseRegistry</t>
+          <t xml:space="preserve">  &gt; tbl_CaseRegistry</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Master Case File Registry — every case, investigation milestones, progress tracking</t>
+          <t>Master Case File Registry - every case, investigation milestones, progress tracking</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1353,12 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_ChainOfCustody</t>
+          <t xml:space="preserve">  &gt; tbl_ChainOfCustody</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Exhibit Chain of Custody — every handover logged</t>
+          <t>Exhibit Chain of Custody - every handover logged</t>
         </is>
       </c>
     </row>
@@ -1372,24 +1372,24 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_CaseFiles</t>
+          <t xml:space="preserve">  &gt; tbl_CaseFiles</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Case File Tracker — DPP submission pipeline, completeness scoring</t>
+          <t>Case File Tracker - DPP submission pipeline, completeness scoring</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_Witnesses</t>
+          <t xml:space="preserve">  &gt; tbl_Witnesses</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Witness &amp; Statement Register — testimony, protection, summons</t>
+          <t>Witness &amp; Statement Register - testimony, protection, summons</t>
         </is>
       </c>
     </row>
@@ -1403,36 +1403,36 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_Personnel</t>
+          <t xml:space="preserve">  &gt; tbl_Personnel</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Personnel Register — staff, qualifications, polygraph</t>
+          <t>Personnel Register - staff, qualifications, polygraph</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; tbl_Vehicles</t>
+          <t xml:space="preserve">  &gt; tbl_Vehicles</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Vehicle/Fleet Log — status, service, fitness</t>
+          <t>Vehicle/Fleet Log - status, service, fitness</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;&gt; Lookups</t>
+          <t xml:space="preserve">  &gt; Lookups</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Reference Data — Jamaica-specific lookups</t>
+          <t>Reference Data - Jamaica-specific lookups</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>CONFIDENTIAL — FOR OFFICIAL USE ONLY | FNID Area 3 | Search warrants under Section 91, Firearms Act 2022</t>
+          <t>CONFIDENTIAL - FOR OFFICIAL USE ONLY | FNID Area 3 | Search warrants under Section 91, Firearms Act 2022</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       <formula>"Cold Case"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="beginsWith" dxfId="3">
-      <formula>"Closed — Convicted"</formula>
+      <formula>"Closed - Convicted"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E1000">
@@ -3976,14 +3976,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>FNID AREA 3 — DAILY COMMAND DASHBOARD</t>
+          <t>FNID AREA 3 - DAILY COMMAND DASHBOARD</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Intelligence → Operations → Seizures → Arrests → Forensics → DPP → Court</t>
+          <t>Intelligence &gt; Operations &gt; Seizures &gt; Arrests &gt; Forensics &gt; DPP &gt; Court</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>→ Converted to Op</t>
+          <t>Converted to Op</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -4066,7 +4066,7 @@
         <v/>
       </c>
       <c r="H6" s="20">
-        <f>IFERROR(COUNTIF(tbl_IntelLog[TriageDecision],"Action*")/(COUNTA(tbl_IntelLog[IntelID])-COUNTBLANK(tbl_IntelLog[IntelID])),"—")</f>
+        <f>IFERROR(COUNTIF(tbl_IntelLog[TriageDecision],"Action*")/(COUNTA(tbl_IntelLog[IntelID])-COUNTBLANK(tbl_IntelLog[IntelID])),"-")</f>
         <v/>
       </c>
     </row>
@@ -4141,15 +4141,15 @@
         <v/>
       </c>
       <c r="F10" s="20">
-        <f>IFERROR(COUNTIF(tbl_Operations[Outcome],"Successful*")/(COUNTA(tbl_Operations[OpsID])-COUNTBLANK(tbl_Operations[OpsID])),"—")</f>
+        <f>IFERROR(COUNTIF(tbl_Operations[Outcome],"Successful*")/(COUNTA(tbl_Operations[OpsID])-COUNTBLANK(tbl_Operations[OpsID])),"-")</f>
         <v/>
       </c>
       <c r="G10" s="20">
-        <f>IFERROR(COUNTIF(tbl_Operations[InspectorPresent],"Yes")/COUNTA(tbl_Operations[InspectorPresent]),"—")</f>
+        <f>IFERROR(COUNTIF(tbl_Operations[InspectorPresent],"Yes")/COUNTA(tbl_Operations[InspectorPresent]),"-")</f>
         <v/>
       </c>
       <c r="H10" s="20">
-        <f>IFERROR(COUNTIF(tbl_Operations[BodyCamActivated],"Yes")/COUNTA(tbl_Operations[BodyCamActivated]),"—")</f>
+        <f>IFERROR(COUNTIF(tbl_Operations[BodyCamActivated],"Yes")/COUNTA(tbl_Operations[BodyCamActivated]),"-")</f>
         <v/>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
         <v/>
       </c>
       <c r="F22" s="20">
-        <f>IFERROR(COUNTIF(tbl_Arrests[48hr_Met],"Yes")/COUNTA(tbl_Arrests[48hr_Met]),"—")</f>
+        <f>IFERROR(COUNTIF(tbl_Arrests[48hr_Met],"Yes")/COUNTA(tbl_Arrests[48hr_Met]),"-")</f>
         <v/>
       </c>
       <c r="G22" s="20">
@@ -4417,12 +4417,12 @@
       </c>
       <c r="B25" s="26" t="inlineStr">
         <is>
-          <t>Open — Active</t>
+          <t>Open - Active</t>
         </is>
       </c>
       <c r="C25" s="26" t="inlineStr">
         <is>
-          <t>Open — Pending</t>
+          <t>Open - Pending</t>
         </is>
       </c>
       <c r="D25" s="26" t="inlineStr">
@@ -4457,11 +4457,11 @@
         <v/>
       </c>
       <c r="B26" s="20">
-        <f>COUNTIF(tbl_CaseRegistry[CaseStatus],"Open — Active*")</f>
+        <f>COUNTIF(tbl_CaseRegistry[CaseStatus],"Open - Active*")</f>
         <v/>
       </c>
       <c r="C26" s="20">
-        <f>COUNTIF(tbl_CaseRegistry[CaseStatus],"Open — Pending*")</f>
+        <f>COUNTIF(tbl_CaseRegistry[CaseStatus],"Open - Pending*")</f>
         <v/>
       </c>
       <c r="D26" s="20">
@@ -4481,7 +4481,7 @@
         <v/>
       </c>
       <c r="H26" s="20">
-        <f>IFERROR(AVERAGE(tbl_CaseRegistry[InvestigationProgress]),"—")</f>
+        <f>IFERROR(AVERAGE(tbl_CaseRegistry[InvestigationProgress]),"-")</f>
         <v/>
       </c>
     </row>
@@ -4560,11 +4560,11 @@
         <v/>
       </c>
       <c r="G30" s="20">
-        <f>IFERROR(AVERAGE(tbl_CaseFiles[FileCompletenessScore]),"—")</f>
+        <f>IFERROR(AVERAGE(tbl_CaseFiles[FileCompletenessScore]),"-")</f>
         <v/>
       </c>
       <c r="H30" s="20">
-        <f>IFERROR(AVERAGE(tbl_CaseFiles[DaysInPipeline]),"—")</f>
+        <f>IFERROR(AVERAGE(tbl_CaseFiles[DaysInPipeline]),"-")</f>
         <v/>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Action — Mount Operation</t>
+          <t>Action - Mount Operation</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4861,12 +4861,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Section 91 — Firearms Act 2022</t>
+          <t>Section 91 - Firearms Act 2022</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Pistol — Semi-Auto</t>
+          <t>Pistol - Semi-Auto</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Cannabis/Ganja — Compressed</t>
+          <t>Cannabis/Ganja - Compressed</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4886,17 +4886,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>s.5 — Possession of Prohibited Weapon (15-25yr)</t>
+          <t>s.5 - Possession of Prohibited Weapon (15-25yr)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Import/Export — Cannabis (DDA Part IIIA)</t>
+          <t>Import/Export - Cannabis (DDA Part IIIA)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Gun Court — High Court Division (judge alone, in camera)</t>
+          <t>Gun Court - High Court Division (judge alone, in camera)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Successful — Seizure + Arrest</t>
+          <t>Successful - Seizure + Arrest</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -4946,7 +4946,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Held — Active Case</t>
+          <t>Held - Active Case</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Open — Active Investigation</t>
+          <t>Open - Active Investigation</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Action — Surveillance</t>
+          <t>Action - Surveillance</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4993,12 +4993,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Section 21 — Dangerous Drugs Act</t>
+          <t>Section 21 - Dangerous Drugs Act</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pistol — Revolver</t>
+          <t>Pistol - Revolver</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Cannabis/Ganja — Loose</t>
+          <t>Cannabis/Ganja - Loose</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5018,17 +5018,17 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>s.6 — Stockpiling (3+ weapons / 50+ rounds)</t>
+          <t>s.6 - Stockpiling (3+ weapons / 50+ rounds)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Import/Export — Cocaine (DDA Part IV)</t>
+          <t>Import/Export - Cocaine (DDA Part IV)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Gun Court — Circuit Court Division (jury, murder/treason)</t>
+          <t>Gun Court - Circuit Court Division (jury, murder/treason)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Successful — Seizure Only</t>
+          <t>Successful - Seizure Only</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -5068,17 +5068,17 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Submitted — Pending</t>
+          <t>Submitted - Pending</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Submitted — Pending</t>
+          <t>Submitted - Pending</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Held — Court Order</t>
+          <t>Held - Court Order</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Open — Pending Forensics</t>
+          <t>Open - Pending Forensics</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Action — Port Alert</t>
+          <t>Action - Port Alert</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5125,12 +5125,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Section 14 — POCA 2007</t>
+          <t>Section 14 - POCA 2007</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Rifle — Semi-Auto</t>
+          <t>Rifle - Semi-Auto</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cannabis/Ganja — Oil/Edibles</t>
+          <t>Cannabis/Ganja - Oil/Edibles</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5150,17 +5150,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>s.7 — Trafficking in Prohibited Weapon (20yr min)</t>
+          <t>s.7 - Trafficking in Prohibited Weapon (20yr min)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Import/Export — Heroin (DDA Part IV)</t>
+          <t>Import/Export - Heroin (DDA Part IV)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Gun Court — RM Division (preliminary exam)</t>
+          <t>Gun Court - RM Division (preliminary exam)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Successful — Arrest Only</t>
+          <t>Successful - Arrest Only</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -5200,12 +5200,12 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Traced — US Origin</t>
+          <t>Traced - US Origin</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Destroyed — Authorized</t>
+          <t>Destroyed - Authorized</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -5220,12 +5220,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Open — Pending Witness Statements</t>
+          <t>Open - Pending Witness Statements</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>Trafficking — Firearms</t>
+          <t>Trafficking - Firearms</t>
         </is>
       </c>
     </row>
@@ -5252,12 +5252,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ZOSO — Warrantless (s.5 ZOSO Act)</t>
+          <t>ZOSO - Warrantless (s.5 ZOSO Act)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Rifle — Bolt Action</t>
+          <t>Rifle - Bolt Action</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5267,7 +5267,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Cocaine — Powder</t>
+          <t>Cocaine - Powder</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -5277,12 +5277,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>s.8 — Possession with Intent to Traffic</t>
+          <t>s.8 - Possession with Intent to Traffic</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Dealing/Trafficking — Cannabis</t>
+          <t>Dealing/Trafficking - Cannabis</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Released — No Charge</t>
+          <t>Released - No Charge</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Partial — Intel Developed</t>
+          <t>Partial - Intel Developed</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -5322,12 +5322,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Hit — Confirmed Match</t>
+          <t>Hit - Confirmed Match</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Traced — Non-US Origin</t>
+          <t>Traced - Non-US Origin</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -5342,17 +5342,17 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Trafficking — Firearms</t>
+          <t>Trafficking - Firearms</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Open — Surveillance</t>
+          <t>Open - Surveillance</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Trafficking — Narcotics</t>
+          <t>Trafficking - Narcotics</t>
         </is>
       </c>
     </row>
@@ -5374,12 +5374,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SOE — Warrantless</t>
+          <t>SOE - Warrantless</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Rifle — Assault</t>
+          <t>Rifle - Assault</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Cocaine — Crack</t>
+          <t>Cocaine - Crack</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5399,12 +5399,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>s.9 — Manufacture of Prohibited Weapon</t>
+          <t>s.9 - Manufacture of Prohibited Weapon</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Dealing/Trafficking — Cocaine</t>
+          <t>Dealing/Trafficking - Cocaine</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Released — Insufficient Evidence</t>
+          <t>Released - Insufficient Evidence</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Negative — No Finds</t>
+          <t>Negative - No Finds</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -5444,17 +5444,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Hit — Unconfirmed</t>
+          <t>Hit - Unconfirmed</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Untraceable — No Serial</t>
+          <t>Untraceable - No Serial</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Forfeited — POCA</t>
+          <t>Forfeited - POCA</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -5464,12 +5464,12 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Trafficking — Narcotics</t>
+          <t>Trafficking - Narcotics</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Open — Pending DPP Submission</t>
+          <t>Open - Pending DPP Submission</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -5521,12 +5521,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>s.10 — Dealing in Prohibited Weapon</t>
+          <t>s.10 - Dealing in Prohibited Weapon</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Dealing/Trafficking — Heroin</t>
+          <t>Dealing/Trafficking - Heroin</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Ruling — Charge Approved</t>
+          <t>Ruling - Charge Approved</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -5556,7 +5556,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Aborted — Compromised</t>
+          <t>Aborted - Compromised</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Untraceable — Obliterated</t>
+          <t>Untraceable - Obliterated</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -5581,12 +5581,12 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Forfeiture Order — Post Conviction</t>
+          <t>Forfeiture Order - Post Conviction</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Trafficking — Multi-Commodity</t>
+          <t>Trafficking - Multi-Commodity</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Intel Filed — Monitor</t>
+          <t>Intel Filed - Monitor</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -5638,12 +5638,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>s.12 — Diversion of Lawful Firearms</t>
+          <t>s.12 - Diversion of Lawful Firearms</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Possession — Cannabis (&gt;2oz)</t>
+          <t>Possession - Cannabis (&gt;2oz)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Ruling — No Charge (Insufficient Evidence)</t>
+          <t>Ruling - No Charge (Insufficient Evidence)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Aborted — Safety Concern</t>
+          <t>Aborted - Safety Concern</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -5693,12 +5693,12 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Closed — Convicted</t>
+          <t>Closed - Convicted</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Import/Export — Narcotics</t>
+          <t>Import/Export - Narcotics</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5710,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Closed — Insufficient Info</t>
+          <t>Closed - Insufficient Info</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5740,12 +5740,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>s.29 — Unmarked Firearm</t>
+          <t>s.29 - Unmarked Firearm</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Possession — Cocaine</t>
+          <t>Possession - Cocaine</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -5780,12 +5780,12 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Closed — Acquitted</t>
+          <t>Closed - Acquitted</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>Import/Export — Firearms</t>
+          <t>Import/Export - Firearms</t>
         </is>
       </c>
     </row>
@@ -5797,7 +5797,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Joint Op — JCA</t>
+          <t>Joint Op - JCA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Cultivation — Cannabis (&gt;5 plants)</t>
+          <t>Cultivation - Cannabis (&gt;5 plants)</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Closed — No Charge (Insufficient Evidence)</t>
+          <t>Closed - No Charge (Insufficient Evidence)</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Joint Op — JDF</t>
+          <t>Joint Op - JDF</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Cultivation — Coca/Opium</t>
+          <t>Cultivation - Coca/Opium</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Closed — Withdrawn</t>
+          <t>Closed - Withdrawn</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Joint Op — MOCA</t>
+          <t>Joint Op - MOCA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Deemed Dealing — School Premises</t>
+          <t>Deemed Dealing - School Premises</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Cold Case — Under Review</t>
+          <t>Cold Case - Under Review</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -5983,12 +5983,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Joint Op — DEA</t>
+          <t>Joint Op - DEA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Component — Frame/Receiver</t>
+          <t>Component - Frame/Receiver</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -5998,7 +5998,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Deemed Dealing — Heroin &gt;1/10oz</t>
+          <t>Deemed Dealing - Heroin &gt;1/10oz</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Cold Case — Dormant</t>
+          <t>Cold Case - Dormant</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
@@ -6035,7 +6035,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Component — Barrel</t>
+          <t>Component - Barrel</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -6055,7 +6055,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Merged — See Linked Case</t>
+          <t>Merged - See Linked Case</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Component — Slide</t>
+          <t>Component - Slide</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">

</xml_diff>

<commit_message>
Fix Excel validation errors - remove duplicate AutoFilter conflict
The workbook was triggering Excel's repair mechanism on every table
because each sheet had both a sheet-level AutoFilter (from
ws.auto_filter.ref in write_headers) AND a Table-level AutoFilter
(built into the Table object). Excel treats this as a conflict and
strips both the AutoFilter and the Table entirely.

Fix: removed ws.auto_filter.ref from write_headers(). Excel Tables
manage their own AutoFilter internally - the sheet-level one was
redundant and caused the "Removed Feature: AutoFilter / Table"
repair warnings on all 13 tables.

Verified via XML inspection:
- Zero sheet-level autoFilters remain
- All 13 table autoFilters match their table refs exactly

https://claude.ai/code/session_01PQmx3HYDSPG2GvHuVy9J6w
</commit_message>
<xml_diff>
--- a/FNID_Area3_Operational_Workbook.xlsx
+++ b/FNID_Area3_Operational_Workbook.xlsx
@@ -24,21 +24,7 @@
     <sheet name="tbl_Personnel" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="tbl_Vehicles" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'tbl_IntelLog'!$A$1:$W$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'tbl_Operations'!$A$1:$AG$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'tbl_FirearmSeizures'!$A$1:$AM$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'tbl_NarcoticSeizures'!$A$1:$AE$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'tbl_OtherSeizures'!$A$1:$U$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'tbl_Arrests'!$A$1:$AJ$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'tbl_CaseRegistry'!$A$1:$AY$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'tbl_ChainOfCustody'!$A$1:$S$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'tbl_CaseFiles'!$A$1:$AI$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'tbl_Witnesses'!$A$1:$V$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'tbl_Informants'!$A$1:$R$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'tbl_Personnel'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'tbl_Vehicles'!$A$1:$O$1</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2118,7 +2104,6 @@
       <c r="AY6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AY1"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="beginsWith" dxfId="1">
       <formula>"Open"</formula>
@@ -2463,7 +2448,6 @@
       <c r="S6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
   <dataValidations count="2">
     <dataValidation sqref="O2:O1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid" error="Select from dropdown" type="list">
       <formula1>=Lookups!$Q$2:$Q$3</formula1>
@@ -2934,7 +2918,6 @@
       <c r="AI6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI1"/>
   <conditionalFormatting sqref="AF2:AF1000">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0.5</formula>
@@ -3250,7 +3233,6 @@
       <c r="V6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V1"/>
   <conditionalFormatting sqref="R2:R1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
@@ -3519,7 +3501,6 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="849B"/>
-  <autoFilter ref="A1:R1"/>
   <conditionalFormatting sqref="N2:N1000">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>=AND(N2&lt;&gt;"",N2&lt;TODAY())</formula>
@@ -3733,7 +3714,6 @@
       <c r="P6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3931,7 +3911,6 @@
       <c r="O6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
   <conditionalFormatting sqref="K2:K1000">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>=AND(K2&lt;&gt;"",K2&lt;TODAY())</formula>
@@ -6450,7 +6429,6 @@
       <c r="W6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W1"/>
   <conditionalFormatting sqref="F2:F1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Critical"</formula>
@@ -6892,7 +6870,6 @@
       <c r="AG6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG1"/>
   <conditionalFormatting sqref="Q2:Q1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"No"</formula>
@@ -7405,7 +7382,6 @@
       <c r="AM6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM1"/>
   <conditionalFormatting sqref="AB2:AB1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Certificate Overdue"</formula>
@@ -7854,7 +7830,6 @@
       <c r="AE6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AE1"/>
   <conditionalFormatting sqref="R2:R1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Certificate Overdue"</formula>
@@ -8167,7 +8142,6 @@
       <c r="U6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U1"/>
   <dataValidations count="1">
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid" error="Select from dropdown" type="list">
       <formula1>=Lookups!$P$2:$P$15</formula1>
@@ -8646,7 +8620,6 @@
       <c r="AJ6" s="33" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ1"/>
   <conditionalFormatting sqref="W2:W1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"BREACH"</formula>

</xml_diff>